<commit_message>
Fix: Modelos de Base de Datos y capturas del prototipo añadidos a la Memoria. Gantt actualizado.
</commit_message>
<xml_diff>
--- a/docs/Diagrama de Gantt.xlsx
+++ b/docs/Diagrama de Gantt.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27D4072D-75AC-4692-A4DE-363BF5A9A3A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25264100-4A71-47A5-829C-0A0BCC17F44B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="0" yWindow="2076" windowWidth="30960" windowHeight="12204" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ProjectSchedule" sheetId="11" r:id="rId1"/>
@@ -1315,23 +1315,23 @@
     <xf numFmtId="168" fontId="9" fillId="0" borderId="2" xfId="10">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="167" fontId="0" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="3" xfId="9" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="8">
       <alignment horizontal="right" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="8" applyBorder="1">
       <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="3" xfId="9" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="54">
@@ -2043,106 +2043,106 @@
         <v>2</v>
       </c>
       <c r="B3" s="51"/>
-      <c r="C3" s="88" t="s">
+      <c r="C3" s="92" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="89"/>
-      <c r="E3" s="93">
+      <c r="D3" s="93"/>
+      <c r="E3" s="91">
         <v>46063</v>
       </c>
-      <c r="F3" s="93"/>
+      <c r="F3" s="91"/>
     </row>
     <row r="4" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="88" t="s">
+      <c r="C4" s="92" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="89"/>
+      <c r="D4" s="93"/>
       <c r="E4" s="7">
         <v>8</v>
       </c>
-      <c r="I4" s="90">
+      <c r="I4" s="88">
         <f>I5</f>
         <v>46111</v>
       </c>
-      <c r="J4" s="91"/>
-      <c r="K4" s="91"/>
-      <c r="L4" s="91"/>
-      <c r="M4" s="91"/>
-      <c r="N4" s="91"/>
-      <c r="O4" s="92"/>
-      <c r="P4" s="90">
+      <c r="J4" s="89"/>
+      <c r="K4" s="89"/>
+      <c r="L4" s="89"/>
+      <c r="M4" s="89"/>
+      <c r="N4" s="89"/>
+      <c r="O4" s="90"/>
+      <c r="P4" s="88">
         <f>P5</f>
         <v>46118</v>
       </c>
-      <c r="Q4" s="91"/>
-      <c r="R4" s="91"/>
-      <c r="S4" s="91"/>
-      <c r="T4" s="91"/>
-      <c r="U4" s="91"/>
-      <c r="V4" s="92"/>
-      <c r="W4" s="90">
+      <c r="Q4" s="89"/>
+      <c r="R4" s="89"/>
+      <c r="S4" s="89"/>
+      <c r="T4" s="89"/>
+      <c r="U4" s="89"/>
+      <c r="V4" s="90"/>
+      <c r="W4" s="88">
         <f>W5</f>
         <v>46125</v>
       </c>
-      <c r="X4" s="91"/>
-      <c r="Y4" s="91"/>
-      <c r="Z4" s="91"/>
-      <c r="AA4" s="91"/>
-      <c r="AB4" s="91"/>
-      <c r="AC4" s="92"/>
-      <c r="AD4" s="90">
+      <c r="X4" s="89"/>
+      <c r="Y4" s="89"/>
+      <c r="Z4" s="89"/>
+      <c r="AA4" s="89"/>
+      <c r="AB4" s="89"/>
+      <c r="AC4" s="90"/>
+      <c r="AD4" s="88">
         <f>AD5</f>
         <v>46132</v>
       </c>
-      <c r="AE4" s="91"/>
-      <c r="AF4" s="91"/>
-      <c r="AG4" s="91"/>
-      <c r="AH4" s="91"/>
-      <c r="AI4" s="91"/>
-      <c r="AJ4" s="92"/>
-      <c r="AK4" s="90">
+      <c r="AE4" s="89"/>
+      <c r="AF4" s="89"/>
+      <c r="AG4" s="89"/>
+      <c r="AH4" s="89"/>
+      <c r="AI4" s="89"/>
+      <c r="AJ4" s="90"/>
+      <c r="AK4" s="88">
         <f>AK5</f>
         <v>46139</v>
       </c>
-      <c r="AL4" s="91"/>
-      <c r="AM4" s="91"/>
-      <c r="AN4" s="91"/>
-      <c r="AO4" s="91"/>
-      <c r="AP4" s="91"/>
-      <c r="AQ4" s="92"/>
-      <c r="AR4" s="90">
+      <c r="AL4" s="89"/>
+      <c r="AM4" s="89"/>
+      <c r="AN4" s="89"/>
+      <c r="AO4" s="89"/>
+      <c r="AP4" s="89"/>
+      <c r="AQ4" s="90"/>
+      <c r="AR4" s="88">
         <f>AR5</f>
         <v>46146</v>
       </c>
-      <c r="AS4" s="91"/>
-      <c r="AT4" s="91"/>
-      <c r="AU4" s="91"/>
-      <c r="AV4" s="91"/>
-      <c r="AW4" s="91"/>
-      <c r="AX4" s="92"/>
-      <c r="AY4" s="90">
+      <c r="AS4" s="89"/>
+      <c r="AT4" s="89"/>
+      <c r="AU4" s="89"/>
+      <c r="AV4" s="89"/>
+      <c r="AW4" s="89"/>
+      <c r="AX4" s="90"/>
+      <c r="AY4" s="88">
         <f>AY5</f>
         <v>46153</v>
       </c>
-      <c r="AZ4" s="91"/>
-      <c r="BA4" s="91"/>
-      <c r="BB4" s="91"/>
-      <c r="BC4" s="91"/>
-      <c r="BD4" s="91"/>
-      <c r="BE4" s="92"/>
-      <c r="BF4" s="90">
+      <c r="AZ4" s="89"/>
+      <c r="BA4" s="89"/>
+      <c r="BB4" s="89"/>
+      <c r="BC4" s="89"/>
+      <c r="BD4" s="89"/>
+      <c r="BE4" s="90"/>
+      <c r="BF4" s="88">
         <f>BF5</f>
         <v>46160</v>
       </c>
-      <c r="BG4" s="91"/>
-      <c r="BH4" s="91"/>
-      <c r="BI4" s="91"/>
-      <c r="BJ4" s="91"/>
-      <c r="BK4" s="91"/>
-      <c r="BL4" s="92"/>
+      <c r="BG4" s="89"/>
+      <c r="BH4" s="89"/>
+      <c r="BI4" s="89"/>
+      <c r="BJ4" s="89"/>
+      <c r="BK4" s="89"/>
+      <c r="BL4" s="90"/>
     </row>
     <row r="5" spans="1:64" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="46" t="s">
@@ -3006,7 +3006,7 @@
       </c>
       <c r="C12" s="53"/>
       <c r="D12" s="17">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E12" s="84">
         <v>46092</v>
@@ -4793,17 +4793,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="AK4:AQ4"/>
+    <mergeCell ref="AR4:AX4"/>
+    <mergeCell ref="AY4:BE4"/>
     <mergeCell ref="BF4:BL4"/>
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="I4:O4"/>
     <mergeCell ref="P4:V4"/>
     <mergeCell ref="W4:AC4"/>
     <mergeCell ref="AD4:AJ4"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="AK4:AQ4"/>
-    <mergeCell ref="AR4:AX4"/>
-    <mergeCell ref="AY4:BE4"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D9 D11:D19 D21:D35">
     <cfRule type="dataBar" priority="22">
@@ -5052,6 +5052,35 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ImageTagsTaxHTField>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="24" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2d714a3296df14eba7a100bb665443ca">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="49549bf45bfbbfb6cffed527380e77e1" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -5339,36 +5368,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC3AD2E1-977A-4D4F-8EE8-D64B5FFADF75}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F80F839-78EF-4FF4-A673-3CC84279C232}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5387,24 +5407,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC3AD2E1-977A-4D4F-8EE8-D64B5FFADF75}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat: Sistema de autenticación completo, enrutamiento por roles y registro de auditoría en BD
- Implementación de login cifrado con SHA-256 a través de login.php.- Enrutamiento automático a vistas adaptadas al rol del usuario.- Temporizador de inactividad de 30 segundos(A falta de seguir actualizandolo).- Sistema de auditoría para registrar accesos en la tabla logs_eventos mediante registro_log.php.
</commit_message>
<xml_diff>
--- a/docs/Diagrama de Gantt.xlsx
+++ b/docs/Diagrama de Gantt.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25264100-4A71-47A5-829C-0A0BCC17F44B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE1C09CC-E75D-455C-8E2F-1A1FF0CA1F2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2061,11 +2061,11 @@
       </c>
       <c r="D4" s="93"/>
       <c r="E4" s="7">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I4" s="88">
         <f>I5</f>
-        <v>46111</v>
+        <v>46090</v>
       </c>
       <c r="J4" s="89"/>
       <c r="K4" s="89"/>
@@ -2075,7 +2075,7 @@
       <c r="O4" s="90"/>
       <c r="P4" s="88">
         <f>P5</f>
-        <v>46118</v>
+        <v>46097</v>
       </c>
       <c r="Q4" s="89"/>
       <c r="R4" s="89"/>
@@ -2085,7 +2085,7 @@
       <c r="V4" s="90"/>
       <c r="W4" s="88">
         <f>W5</f>
-        <v>46125</v>
+        <v>46104</v>
       </c>
       <c r="X4" s="89"/>
       <c r="Y4" s="89"/>
@@ -2095,7 +2095,7 @@
       <c r="AC4" s="90"/>
       <c r="AD4" s="88">
         <f>AD5</f>
-        <v>46132</v>
+        <v>46111</v>
       </c>
       <c r="AE4" s="89"/>
       <c r="AF4" s="89"/>
@@ -2105,7 +2105,7 @@
       <c r="AJ4" s="90"/>
       <c r="AK4" s="88">
         <f>AK5</f>
-        <v>46139</v>
+        <v>46118</v>
       </c>
       <c r="AL4" s="89"/>
       <c r="AM4" s="89"/>
@@ -2115,7 +2115,7 @@
       <c r="AQ4" s="90"/>
       <c r="AR4" s="88">
         <f>AR5</f>
-        <v>46146</v>
+        <v>46125</v>
       </c>
       <c r="AS4" s="89"/>
       <c r="AT4" s="89"/>
@@ -2125,7 +2125,7 @@
       <c r="AX4" s="90"/>
       <c r="AY4" s="88">
         <f>AY5</f>
-        <v>46153</v>
+        <v>46132</v>
       </c>
       <c r="AZ4" s="89"/>
       <c r="BA4" s="89"/>
@@ -2135,7 +2135,7 @@
       <c r="BE4" s="90"/>
       <c r="BF4" s="88">
         <f>BF5</f>
-        <v>46160</v>
+        <v>46139</v>
       </c>
       <c r="BG4" s="89"/>
       <c r="BH4" s="89"/>
@@ -2156,227 +2156,227 @@
       <c r="G5" s="66"/>
       <c r="I5" s="81">
         <f>Inicio_del_proyecto-WEEKDAY(Inicio_del_proyecto,1)+2+7*(Semana_para_mostrar-1)</f>
-        <v>46111</v>
+        <v>46090</v>
       </c>
       <c r="J5" s="82">
         <f>I5+1</f>
-        <v>46112</v>
+        <v>46091</v>
       </c>
       <c r="K5" s="82">
         <f t="shared" ref="K5:AX5" si="0">J5+1</f>
-        <v>46113</v>
+        <v>46092</v>
       </c>
       <c r="L5" s="82">
         <f t="shared" si="0"/>
-        <v>46114</v>
+        <v>46093</v>
       </c>
       <c r="M5" s="82">
         <f t="shared" si="0"/>
-        <v>46115</v>
+        <v>46094</v>
       </c>
       <c r="N5" s="82">
         <f t="shared" si="0"/>
-        <v>46116</v>
+        <v>46095</v>
       </c>
       <c r="O5" s="83">
         <f t="shared" si="0"/>
-        <v>46117</v>
+        <v>46096</v>
       </c>
       <c r="P5" s="81">
         <f>O5+1</f>
-        <v>46118</v>
+        <v>46097</v>
       </c>
       <c r="Q5" s="82">
         <f>P5+1</f>
-        <v>46119</v>
+        <v>46098</v>
       </c>
       <c r="R5" s="82">
         <f t="shared" si="0"/>
-        <v>46120</v>
+        <v>46099</v>
       </c>
       <c r="S5" s="82">
         <f t="shared" si="0"/>
-        <v>46121</v>
+        <v>46100</v>
       </c>
       <c r="T5" s="82">
         <f t="shared" si="0"/>
-        <v>46122</v>
+        <v>46101</v>
       </c>
       <c r="U5" s="82">
         <f t="shared" si="0"/>
-        <v>46123</v>
+        <v>46102</v>
       </c>
       <c r="V5" s="83">
         <f t="shared" si="0"/>
-        <v>46124</v>
+        <v>46103</v>
       </c>
       <c r="W5" s="81">
         <f>V5+1</f>
-        <v>46125</v>
+        <v>46104</v>
       </c>
       <c r="X5" s="82">
         <f>W5+1</f>
-        <v>46126</v>
+        <v>46105</v>
       </c>
       <c r="Y5" s="82">
         <f t="shared" si="0"/>
-        <v>46127</v>
+        <v>46106</v>
       </c>
       <c r="Z5" s="82">
         <f t="shared" si="0"/>
-        <v>46128</v>
+        <v>46107</v>
       </c>
       <c r="AA5" s="82">
         <f t="shared" si="0"/>
-        <v>46129</v>
+        <v>46108</v>
       </c>
       <c r="AB5" s="82">
         <f t="shared" si="0"/>
-        <v>46130</v>
+        <v>46109</v>
       </c>
       <c r="AC5" s="83">
         <f t="shared" si="0"/>
-        <v>46131</v>
+        <v>46110</v>
       </c>
       <c r="AD5" s="81">
         <f>AC5+1</f>
-        <v>46132</v>
+        <v>46111</v>
       </c>
       <c r="AE5" s="82">
         <f>AD5+1</f>
-        <v>46133</v>
+        <v>46112</v>
       </c>
       <c r="AF5" s="82">
         <f t="shared" si="0"/>
-        <v>46134</v>
+        <v>46113</v>
       </c>
       <c r="AG5" s="82">
         <f t="shared" si="0"/>
-        <v>46135</v>
+        <v>46114</v>
       </c>
       <c r="AH5" s="82">
         <f t="shared" si="0"/>
-        <v>46136</v>
+        <v>46115</v>
       </c>
       <c r="AI5" s="82">
         <f t="shared" si="0"/>
-        <v>46137</v>
+        <v>46116</v>
       </c>
       <c r="AJ5" s="83">
         <f t="shared" si="0"/>
-        <v>46138</v>
+        <v>46117</v>
       </c>
       <c r="AK5" s="81">
         <f>AJ5+1</f>
-        <v>46139</v>
+        <v>46118</v>
       </c>
       <c r="AL5" s="82">
         <f>AK5+1</f>
-        <v>46140</v>
+        <v>46119</v>
       </c>
       <c r="AM5" s="82">
         <f t="shared" si="0"/>
-        <v>46141</v>
+        <v>46120</v>
       </c>
       <c r="AN5" s="82">
         <f t="shared" si="0"/>
-        <v>46142</v>
+        <v>46121</v>
       </c>
       <c r="AO5" s="82">
         <f t="shared" si="0"/>
-        <v>46143</v>
+        <v>46122</v>
       </c>
       <c r="AP5" s="82">
         <f t="shared" si="0"/>
-        <v>46144</v>
+        <v>46123</v>
       </c>
       <c r="AQ5" s="83">
         <f t="shared" si="0"/>
-        <v>46145</v>
+        <v>46124</v>
       </c>
       <c r="AR5" s="81">
         <f>AQ5+1</f>
-        <v>46146</v>
+        <v>46125</v>
       </c>
       <c r="AS5" s="82">
         <f>AR5+1</f>
-        <v>46147</v>
+        <v>46126</v>
       </c>
       <c r="AT5" s="82">
         <f t="shared" si="0"/>
-        <v>46148</v>
+        <v>46127</v>
       </c>
       <c r="AU5" s="82">
         <f t="shared" si="0"/>
-        <v>46149</v>
+        <v>46128</v>
       </c>
       <c r="AV5" s="82">
         <f t="shared" si="0"/>
-        <v>46150</v>
+        <v>46129</v>
       </c>
       <c r="AW5" s="82">
         <f t="shared" si="0"/>
-        <v>46151</v>
+        <v>46130</v>
       </c>
       <c r="AX5" s="83">
         <f t="shared" si="0"/>
-        <v>46152</v>
+        <v>46131</v>
       </c>
       <c r="AY5" s="81">
         <f>AX5+1</f>
-        <v>46153</v>
+        <v>46132</v>
       </c>
       <c r="AZ5" s="82">
         <f>AY5+1</f>
-        <v>46154</v>
+        <v>46133</v>
       </c>
       <c r="BA5" s="82">
         <f t="shared" ref="BA5:BE5" si="1">AZ5+1</f>
-        <v>46155</v>
+        <v>46134</v>
       </c>
       <c r="BB5" s="82">
         <f t="shared" si="1"/>
-        <v>46156</v>
+        <v>46135</v>
       </c>
       <c r="BC5" s="82">
         <f t="shared" si="1"/>
-        <v>46157</v>
+        <v>46136</v>
       </c>
       <c r="BD5" s="82">
         <f t="shared" si="1"/>
-        <v>46158</v>
+        <v>46137</v>
       </c>
       <c r="BE5" s="83">
         <f t="shared" si="1"/>
-        <v>46159</v>
+        <v>46138</v>
       </c>
       <c r="BF5" s="81">
         <f>BE5+1</f>
-        <v>46160</v>
+        <v>46139</v>
       </c>
       <c r="BG5" s="82">
         <f>BF5+1</f>
-        <v>46161</v>
+        <v>46140</v>
       </c>
       <c r="BH5" s="82">
         <f t="shared" ref="BH5:BL5" si="2">BG5+1</f>
-        <v>46162</v>
+        <v>46141</v>
       </c>
       <c r="BI5" s="82">
         <f t="shared" si="2"/>
-        <v>46163</v>
+        <v>46142</v>
       </c>
       <c r="BJ5" s="82">
         <f t="shared" si="2"/>
-        <v>46164</v>
+        <v>46143</v>
       </c>
       <c r="BK5" s="82">
         <f t="shared" si="2"/>
-        <v>46165</v>
+        <v>46144</v>
       </c>
       <c r="BL5" s="83">
         <f t="shared" si="2"/>
-        <v>46166</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="6" spans="1:64" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C13" s="53"/>
       <c r="D13" s="17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E13" s="84">
         <v>46096</v>
@@ -3302,7 +3302,7 @@
       </c>
       <c r="C16" s="55"/>
       <c r="D16" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16" s="85">
         <v>46097</v>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C19" s="55"/>
       <c r="D19" s="20">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="E19" s="85">
         <v>46122</v>

</xml_diff>

<commit_message>
borrador final TFG: Modelo BD en singular, diagramas UX y evidencias añadidas en memoria
</commit_message>
<xml_diff>
--- a/docs/Diagrama de Gantt.xlsx
+++ b/docs/Diagrama de Gantt.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE1C09CC-E75D-455C-8E2F-1A1FF0CA1F2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FE0B9D7-D338-4A25-87BC-98530F3FF03B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -252,13 +252,13 @@
     <t>Diseño Adaptativo Interfaz UCI</t>
   </si>
   <si>
-    <t>Automatización Ahorro Energético (Auto-apagado)</t>
-  </si>
-  <si>
     <t>Redacción de Memoria (Borrador Completo)</t>
   </si>
   <si>
     <t>Control HW 1 (Vídeo Evertz, Luces ETC y Proyección)</t>
+  </si>
+  <si>
+    <t>Automatización cierre de sesion automático</t>
   </si>
 </sst>
 </file>
@@ -2061,11 +2061,11 @@
       </c>
       <c r="D4" s="93"/>
       <c r="E4" s="7">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I4" s="88">
         <f>I5</f>
-        <v>46090</v>
+        <v>46111</v>
       </c>
       <c r="J4" s="89"/>
       <c r="K4" s="89"/>
@@ -2075,7 +2075,7 @@
       <c r="O4" s="90"/>
       <c r="P4" s="88">
         <f>P5</f>
-        <v>46097</v>
+        <v>46118</v>
       </c>
       <c r="Q4" s="89"/>
       <c r="R4" s="89"/>
@@ -2085,7 +2085,7 @@
       <c r="V4" s="90"/>
       <c r="W4" s="88">
         <f>W5</f>
-        <v>46104</v>
+        <v>46125</v>
       </c>
       <c r="X4" s="89"/>
       <c r="Y4" s="89"/>
@@ -2095,7 +2095,7 @@
       <c r="AC4" s="90"/>
       <c r="AD4" s="88">
         <f>AD5</f>
-        <v>46111</v>
+        <v>46132</v>
       </c>
       <c r="AE4" s="89"/>
       <c r="AF4" s="89"/>
@@ -2105,7 +2105,7 @@
       <c r="AJ4" s="90"/>
       <c r="AK4" s="88">
         <f>AK5</f>
-        <v>46118</v>
+        <v>46139</v>
       </c>
       <c r="AL4" s="89"/>
       <c r="AM4" s="89"/>
@@ -2115,7 +2115,7 @@
       <c r="AQ4" s="90"/>
       <c r="AR4" s="88">
         <f>AR5</f>
-        <v>46125</v>
+        <v>46146</v>
       </c>
       <c r="AS4" s="89"/>
       <c r="AT4" s="89"/>
@@ -2125,7 +2125,7 @@
       <c r="AX4" s="90"/>
       <c r="AY4" s="88">
         <f>AY5</f>
-        <v>46132</v>
+        <v>46153</v>
       </c>
       <c r="AZ4" s="89"/>
       <c r="BA4" s="89"/>
@@ -2135,7 +2135,7 @@
       <c r="BE4" s="90"/>
       <c r="BF4" s="88">
         <f>BF5</f>
-        <v>46139</v>
+        <v>46160</v>
       </c>
       <c r="BG4" s="89"/>
       <c r="BH4" s="89"/>
@@ -2156,227 +2156,227 @@
       <c r="G5" s="66"/>
       <c r="I5" s="81">
         <f>Inicio_del_proyecto-WEEKDAY(Inicio_del_proyecto,1)+2+7*(Semana_para_mostrar-1)</f>
-        <v>46090</v>
+        <v>46111</v>
       </c>
       <c r="J5" s="82">
         <f>I5+1</f>
-        <v>46091</v>
+        <v>46112</v>
       </c>
       <c r="K5" s="82">
         <f t="shared" ref="K5:AX5" si="0">J5+1</f>
-        <v>46092</v>
+        <v>46113</v>
       </c>
       <c r="L5" s="82">
         <f t="shared" si="0"/>
-        <v>46093</v>
+        <v>46114</v>
       </c>
       <c r="M5" s="82">
         <f t="shared" si="0"/>
-        <v>46094</v>
+        <v>46115</v>
       </c>
       <c r="N5" s="82">
         <f t="shared" si="0"/>
-        <v>46095</v>
+        <v>46116</v>
       </c>
       <c r="O5" s="83">
         <f t="shared" si="0"/>
-        <v>46096</v>
+        <v>46117</v>
       </c>
       <c r="P5" s="81">
         <f>O5+1</f>
-        <v>46097</v>
+        <v>46118</v>
       </c>
       <c r="Q5" s="82">
         <f>P5+1</f>
-        <v>46098</v>
+        <v>46119</v>
       </c>
       <c r="R5" s="82">
         <f t="shared" si="0"/>
-        <v>46099</v>
+        <v>46120</v>
       </c>
       <c r="S5" s="82">
         <f t="shared" si="0"/>
-        <v>46100</v>
+        <v>46121</v>
       </c>
       <c r="T5" s="82">
         <f t="shared" si="0"/>
-        <v>46101</v>
+        <v>46122</v>
       </c>
       <c r="U5" s="82">
         <f t="shared" si="0"/>
-        <v>46102</v>
+        <v>46123</v>
       </c>
       <c r="V5" s="83">
         <f t="shared" si="0"/>
-        <v>46103</v>
+        <v>46124</v>
       </c>
       <c r="W5" s="81">
         <f>V5+1</f>
-        <v>46104</v>
+        <v>46125</v>
       </c>
       <c r="X5" s="82">
         <f>W5+1</f>
-        <v>46105</v>
+        <v>46126</v>
       </c>
       <c r="Y5" s="82">
         <f t="shared" si="0"/>
-        <v>46106</v>
+        <v>46127</v>
       </c>
       <c r="Z5" s="82">
         <f t="shared" si="0"/>
-        <v>46107</v>
+        <v>46128</v>
       </c>
       <c r="AA5" s="82">
         <f t="shared" si="0"/>
-        <v>46108</v>
+        <v>46129</v>
       </c>
       <c r="AB5" s="82">
         <f t="shared" si="0"/>
-        <v>46109</v>
+        <v>46130</v>
       </c>
       <c r="AC5" s="83">
         <f t="shared" si="0"/>
-        <v>46110</v>
+        <v>46131</v>
       </c>
       <c r="AD5" s="81">
         <f>AC5+1</f>
-        <v>46111</v>
+        <v>46132</v>
       </c>
       <c r="AE5" s="82">
         <f>AD5+1</f>
-        <v>46112</v>
+        <v>46133</v>
       </c>
       <c r="AF5" s="82">
         <f t="shared" si="0"/>
-        <v>46113</v>
+        <v>46134</v>
       </c>
       <c r="AG5" s="82">
         <f t="shared" si="0"/>
-        <v>46114</v>
+        <v>46135</v>
       </c>
       <c r="AH5" s="82">
         <f t="shared" si="0"/>
-        <v>46115</v>
+        <v>46136</v>
       </c>
       <c r="AI5" s="82">
         <f t="shared" si="0"/>
-        <v>46116</v>
+        <v>46137</v>
       </c>
       <c r="AJ5" s="83">
         <f t="shared" si="0"/>
-        <v>46117</v>
+        <v>46138</v>
       </c>
       <c r="AK5" s="81">
         <f>AJ5+1</f>
-        <v>46118</v>
+        <v>46139</v>
       </c>
       <c r="AL5" s="82">
         <f>AK5+1</f>
-        <v>46119</v>
+        <v>46140</v>
       </c>
       <c r="AM5" s="82">
         <f t="shared" si="0"/>
-        <v>46120</v>
+        <v>46141</v>
       </c>
       <c r="AN5" s="82">
         <f t="shared" si="0"/>
-        <v>46121</v>
+        <v>46142</v>
       </c>
       <c r="AO5" s="82">
         <f t="shared" si="0"/>
-        <v>46122</v>
+        <v>46143</v>
       </c>
       <c r="AP5" s="82">
         <f t="shared" si="0"/>
-        <v>46123</v>
+        <v>46144</v>
       </c>
       <c r="AQ5" s="83">
         <f t="shared" si="0"/>
-        <v>46124</v>
+        <v>46145</v>
       </c>
       <c r="AR5" s="81">
         <f>AQ5+1</f>
-        <v>46125</v>
+        <v>46146</v>
       </c>
       <c r="AS5" s="82">
         <f>AR5+1</f>
-        <v>46126</v>
+        <v>46147</v>
       </c>
       <c r="AT5" s="82">
         <f t="shared" si="0"/>
-        <v>46127</v>
+        <v>46148</v>
       </c>
       <c r="AU5" s="82">
         <f t="shared" si="0"/>
-        <v>46128</v>
+        <v>46149</v>
       </c>
       <c r="AV5" s="82">
         <f t="shared" si="0"/>
-        <v>46129</v>
+        <v>46150</v>
       </c>
       <c r="AW5" s="82">
         <f t="shared" si="0"/>
-        <v>46130</v>
+        <v>46151</v>
       </c>
       <c r="AX5" s="83">
         <f t="shared" si="0"/>
-        <v>46131</v>
+        <v>46152</v>
       </c>
       <c r="AY5" s="81">
         <f>AX5+1</f>
-        <v>46132</v>
+        <v>46153</v>
       </c>
       <c r="AZ5" s="82">
         <f>AY5+1</f>
-        <v>46133</v>
+        <v>46154</v>
       </c>
       <c r="BA5" s="82">
         <f t="shared" ref="BA5:BE5" si="1">AZ5+1</f>
-        <v>46134</v>
+        <v>46155</v>
       </c>
       <c r="BB5" s="82">
         <f t="shared" si="1"/>
-        <v>46135</v>
+        <v>46156</v>
       </c>
       <c r="BC5" s="82">
         <f t="shared" si="1"/>
-        <v>46136</v>
+        <v>46157</v>
       </c>
       <c r="BD5" s="82">
         <f t="shared" si="1"/>
-        <v>46137</v>
+        <v>46158</v>
       </c>
       <c r="BE5" s="83">
         <f t="shared" si="1"/>
-        <v>46138</v>
+        <v>46159</v>
       </c>
       <c r="BF5" s="81">
         <f>BE5+1</f>
-        <v>46139</v>
+        <v>46160</v>
       </c>
       <c r="BG5" s="82">
         <f>BF5+1</f>
-        <v>46140</v>
+        <v>46161</v>
       </c>
       <c r="BH5" s="82">
         <f t="shared" ref="BH5:BL5" si="2">BG5+1</f>
-        <v>46141</v>
+        <v>46162</v>
       </c>
       <c r="BI5" s="82">
         <f t="shared" si="2"/>
-        <v>46142</v>
+        <v>46163</v>
       </c>
       <c r="BJ5" s="82">
         <f t="shared" si="2"/>
-        <v>46143</v>
+        <v>46164</v>
       </c>
       <c r="BK5" s="82">
         <f t="shared" si="2"/>
-        <v>46144</v>
+        <v>46165</v>
       </c>
       <c r="BL5" s="83">
         <f t="shared" si="2"/>
-        <v>46145</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="6" spans="1:64" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3375,11 +3375,11 @@
     <row r="17" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="45"/>
       <c r="B17" s="62" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C17" s="55"/>
       <c r="D17" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E17" s="85">
         <v>46104</v>
@@ -3456,7 +3456,7 @@
       </c>
       <c r="C18" s="55"/>
       <c r="D18" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E18" s="85">
         <v>46115</v>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C19" s="55"/>
       <c r="D19" s="20">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="E19" s="85">
         <v>46122</v>
@@ -3610,7 +3610,7 @@
       </c>
       <c r="C20" s="55"/>
       <c r="D20" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" s="85">
         <v>46129</v>
@@ -3684,7 +3684,7 @@
       </c>
       <c r="C21" s="55"/>
       <c r="D21" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E21" s="85">
         <v>46137</v>
@@ -3834,7 +3834,7 @@
       </c>
       <c r="C23" s="57"/>
       <c r="D23" s="23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E23" s="76">
         <v>46138</v>
@@ -3907,11 +3907,11 @@
     <row r="24" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="45"/>
       <c r="B24" s="63" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C24" s="57"/>
       <c r="D24" s="23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24" s="76">
         <v>46145</v>
@@ -3984,11 +3984,11 @@
     <row r="25" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="45"/>
       <c r="B25" s="63" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C25" s="57"/>
       <c r="D25" s="23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E25" s="76">
         <v>46138</v>

</xml_diff>

<commit_message>
Entrega final: Memoria del TFG finalizada y corregida
</commit_message>
<xml_diff>
--- a/docs/Diagrama de Gantt.xlsx
+++ b/docs/Diagrama de Gantt.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FE0B9D7-D338-4A25-87BC-98530F3FF03B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B507FB0-B91B-4775-86B8-7448F77B04D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1315,6 +1315,12 @@
     <xf numFmtId="168" fontId="9" fillId="0" borderId="2" xfId="10">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="8">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="8" applyBorder="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
     <xf numFmtId="167" fontId="0" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -1326,12 +1332,6 @@
     </xf>
     <xf numFmtId="166" fontId="9" fillId="0" borderId="3" xfId="9" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="8">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="8" applyBorder="1">
-      <alignment horizontal="right" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="54">
@@ -2043,106 +2043,106 @@
         <v>2</v>
       </c>
       <c r="B3" s="51"/>
-      <c r="C3" s="92" t="s">
+      <c r="C3" s="88" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="93"/>
-      <c r="E3" s="91">
+      <c r="D3" s="89"/>
+      <c r="E3" s="93">
         <v>46063</v>
       </c>
-      <c r="F3" s="91"/>
+      <c r="F3" s="93"/>
     </row>
     <row r="4" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="92" t="s">
+      <c r="C4" s="88" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="93"/>
+      <c r="D4" s="89"/>
       <c r="E4" s="7">
         <v>8</v>
       </c>
-      <c r="I4" s="88">
+      <c r="I4" s="90">
         <f>I5</f>
         <v>46111</v>
       </c>
-      <c r="J4" s="89"/>
-      <c r="K4" s="89"/>
-      <c r="L4" s="89"/>
-      <c r="M4" s="89"/>
-      <c r="N4" s="89"/>
-      <c r="O4" s="90"/>
-      <c r="P4" s="88">
+      <c r="J4" s="91"/>
+      <c r="K4" s="91"/>
+      <c r="L4" s="91"/>
+      <c r="M4" s="91"/>
+      <c r="N4" s="91"/>
+      <c r="O4" s="92"/>
+      <c r="P4" s="90">
         <f>P5</f>
         <v>46118</v>
       </c>
-      <c r="Q4" s="89"/>
-      <c r="R4" s="89"/>
-      <c r="S4" s="89"/>
-      <c r="T4" s="89"/>
-      <c r="U4" s="89"/>
-      <c r="V4" s="90"/>
-      <c r="W4" s="88">
+      <c r="Q4" s="91"/>
+      <c r="R4" s="91"/>
+      <c r="S4" s="91"/>
+      <c r="T4" s="91"/>
+      <c r="U4" s="91"/>
+      <c r="V4" s="92"/>
+      <c r="W4" s="90">
         <f>W5</f>
         <v>46125</v>
       </c>
-      <c r="X4" s="89"/>
-      <c r="Y4" s="89"/>
-      <c r="Z4" s="89"/>
-      <c r="AA4" s="89"/>
-      <c r="AB4" s="89"/>
-      <c r="AC4" s="90"/>
-      <c r="AD4" s="88">
+      <c r="X4" s="91"/>
+      <c r="Y4" s="91"/>
+      <c r="Z4" s="91"/>
+      <c r="AA4" s="91"/>
+      <c r="AB4" s="91"/>
+      <c r="AC4" s="92"/>
+      <c r="AD4" s="90">
         <f>AD5</f>
         <v>46132</v>
       </c>
-      <c r="AE4" s="89"/>
-      <c r="AF4" s="89"/>
-      <c r="AG4" s="89"/>
-      <c r="AH4" s="89"/>
-      <c r="AI4" s="89"/>
-      <c r="AJ4" s="90"/>
-      <c r="AK4" s="88">
+      <c r="AE4" s="91"/>
+      <c r="AF4" s="91"/>
+      <c r="AG4" s="91"/>
+      <c r="AH4" s="91"/>
+      <c r="AI4" s="91"/>
+      <c r="AJ4" s="92"/>
+      <c r="AK4" s="90">
         <f>AK5</f>
         <v>46139</v>
       </c>
-      <c r="AL4" s="89"/>
-      <c r="AM4" s="89"/>
-      <c r="AN4" s="89"/>
-      <c r="AO4" s="89"/>
-      <c r="AP4" s="89"/>
-      <c r="AQ4" s="90"/>
-      <c r="AR4" s="88">
+      <c r="AL4" s="91"/>
+      <c r="AM4" s="91"/>
+      <c r="AN4" s="91"/>
+      <c r="AO4" s="91"/>
+      <c r="AP4" s="91"/>
+      <c r="AQ4" s="92"/>
+      <c r="AR4" s="90">
         <f>AR5</f>
         <v>46146</v>
       </c>
-      <c r="AS4" s="89"/>
-      <c r="AT4" s="89"/>
-      <c r="AU4" s="89"/>
-      <c r="AV4" s="89"/>
-      <c r="AW4" s="89"/>
-      <c r="AX4" s="90"/>
-      <c r="AY4" s="88">
+      <c r="AS4" s="91"/>
+      <c r="AT4" s="91"/>
+      <c r="AU4" s="91"/>
+      <c r="AV4" s="91"/>
+      <c r="AW4" s="91"/>
+      <c r="AX4" s="92"/>
+      <c r="AY4" s="90">
         <f>AY5</f>
         <v>46153</v>
       </c>
-      <c r="AZ4" s="89"/>
-      <c r="BA4" s="89"/>
-      <c r="BB4" s="89"/>
-      <c r="BC4" s="89"/>
-      <c r="BD4" s="89"/>
-      <c r="BE4" s="90"/>
-      <c r="BF4" s="88">
+      <c r="AZ4" s="91"/>
+      <c r="BA4" s="91"/>
+      <c r="BB4" s="91"/>
+      <c r="BC4" s="91"/>
+      <c r="BD4" s="91"/>
+      <c r="BE4" s="92"/>
+      <c r="BF4" s="90">
         <f>BF5</f>
         <v>46160</v>
       </c>
-      <c r="BG4" s="89"/>
-      <c r="BH4" s="89"/>
-      <c r="BI4" s="89"/>
-      <c r="BJ4" s="89"/>
-      <c r="BK4" s="89"/>
-      <c r="BL4" s="90"/>
+      <c r="BG4" s="91"/>
+      <c r="BH4" s="91"/>
+      <c r="BI4" s="91"/>
+      <c r="BJ4" s="91"/>
+      <c r="BK4" s="91"/>
+      <c r="BL4" s="92"/>
     </row>
     <row r="5" spans="1:64" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="46" t="s">
@@ -4065,7 +4065,7 @@
       </c>
       <c r="C26" s="57"/>
       <c r="D26" s="23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E26" s="76">
         <v>46152</v>
@@ -4283,7 +4283,9 @@
         <v>48</v>
       </c>
       <c r="C29" s="59"/>
-      <c r="D29" s="26"/>
+      <c r="D29" s="26">
+        <v>1</v>
+      </c>
       <c r="E29" s="86">
         <v>46153</v>
       </c>
@@ -4358,7 +4360,9 @@
         <v>49</v>
       </c>
       <c r="C30" s="59"/>
-      <c r="D30" s="26"/>
+      <c r="D30" s="26">
+        <v>1</v>
+      </c>
       <c r="E30" s="86">
         <v>46161</v>
       </c>
@@ -4433,7 +4437,9 @@
         <v>50</v>
       </c>
       <c r="C31" s="59"/>
-      <c r="D31" s="26"/>
+      <c r="D31" s="26">
+        <v>1</v>
+      </c>
       <c r="E31" s="86">
         <v>46163</v>
       </c>
@@ -4793,17 +4799,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="AK4:AQ4"/>
-    <mergeCell ref="AR4:AX4"/>
-    <mergeCell ref="AY4:BE4"/>
     <mergeCell ref="BF4:BL4"/>
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="I4:O4"/>
     <mergeCell ref="P4:V4"/>
     <mergeCell ref="W4:AC4"/>
     <mergeCell ref="AD4:AJ4"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="AK4:AQ4"/>
+    <mergeCell ref="AR4:AX4"/>
+    <mergeCell ref="AY4:BE4"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D9 D11:D19 D21:D35">
     <cfRule type="dataBar" priority="22">
@@ -5052,35 +5058,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="24" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2d714a3296df14eba7a100bb665443ca">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="49549bf45bfbbfb6cffed527380e77e1" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -5368,27 +5345,36 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC3AD2E1-977A-4D4F-8EE8-D64B5FFADF75}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ImageTagsTaxHTField>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F80F839-78EF-4FF4-A673-3CC84279C232}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5407,4 +5393,24 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC3AD2E1-977A-4D4F-8EE8-D64B5FFADF75}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>